<commit_message>
Fresh walkgrid scope sheet, decision log, budgets for the reference machine, M0 plan
The Voxistics scope sheet moves to docs/voxistics/. Baseline recorded:
native tests pass, shader check clean, MinGW cross-compile builds.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -546,7 +546,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Voxistics scope (MoSCoW)</t>
+          <t>walkgrid scope (MoSCoW)</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Horizon (edit this): the next playable build -- a world you can build in, decorate and hear, with item logistics decided.</t>
+          <t>Horizon (edit this): the first functional test -- walk a faceted, textured, lit world, hear footsteps with the music, place and remove ground, at 60 fps or better on the owner's PC.</t>
         </is>
       </c>
     </row>
@@ -705,17 +705,17 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>W001</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Engine</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Chunked world, streaming, eviction, regeneration</t>
+          <t>Engine review, prototype outline, foundations</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -728,10 +728,14 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>docs/ENGINE_REVIEW.md, PROTOTYPE_OUTLINE.md, FOUNDATIONS.md</t>
+        </is>
+      </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Part II</t>
+          <t>Foundations</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -743,17 +747,17 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>W002</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Engine</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Save/load: slots, autosave, backups, settings file</t>
+          <t>Plan, approve, build, check; say plainly what wasn't verified</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -763,13 +767,17 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Standing rule, never 'done'</t>
+        </is>
+      </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Part VII</t>
+          <t>Foundations 1</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -781,7 +789,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>W003</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -791,7 +799,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Native tests + frame profiler (F3)</t>
+          <t>Carry the Voxistics engine across intact; take only the Voxistics game layer off (M0)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -801,17 +809,17 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Every change keeps tests at zero failures</t>
+          <t>Frames before and after must match, minus removed features</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Parts XVI-XVII</t>
+          <t>Engine review 3</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -823,7 +831,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>W004</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -833,7 +841,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Lagless rule: cost scales with what's on screen or changing</t>
+          <t>Lots of action without lag: cost scales with what's on screen or changing</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -853,7 +861,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Foundations 4</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -865,7 +873,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>W005</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -875,12 +883,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Release-build performance check on the owner's PC</t>
+          <t>60 fps floor; higher where the machine allows, with no jitter (interpolated rendering)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -890,34 +898,34 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>The Ctrl+F3 report tool exists (perf_report.txt); running the check awaits the owner</t>
+          <t>Checklist T12, T13</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Part XVI</t>
+          <t>Outline D10</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>W006</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Block registry, shapes, 32 px materials with normal/shine/glow maps</t>
+          <t>Working name walkgrid: project, window, save folder</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -927,17 +935,17 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>32 px chosen by owner</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>4.3, 4.13</t>
+          <t>Outline D11</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -949,17 +957,17 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>W007</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Natural, dark, genesis and custodian material sets</t>
+          <t>Layer rule plus tools/check_layers.sh</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -969,13 +977,17 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Approved with the foundations</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>Foundations 2</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -987,17 +999,17 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>W008</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Plant cards</t>
+          <t>Thread model: main thread owns world and graphics; 2 job threads build from copies; version stamps</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1007,13 +1019,17 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Approved with the foundations</t>
+        </is>
+      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>Foundations 3</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -1025,17 +1041,17 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>W009</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Faceted props + dwelling/industry pieces (40 blocks)</t>
+          <t>Fresh walkgrid save format v1 (no Voxistics loaders)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1045,17 +1061,17 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>In the library only, not world gen yet</t>
+          <t>Approved with the foundations</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>Foundations 5</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -1067,17 +1083,17 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>W010</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Try the library out in the landscape</t>
+          <t>Camera-relative rendering (no jitter far from the start)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1087,17 +1103,17 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Owner play-test; decides names and what stays</t>
+          <t>Approved with the foundations</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>Foundations 4.2</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -1109,22 +1125,22 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>W011</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Name pass over all blocks</t>
+          <t>Budgets per frame shown in F3</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1134,12 +1150,12 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>After the landscape try-out</t>
+          <t>Numbers are conservative assumptions; tuned only from reports the owner chooses to share</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Part VIII</t>
+          <t>Foundations 4</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -1151,37 +1167,37 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>W012</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>World</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Landmark shapes: canopy cap, coil stalk</t>
+          <t>Faceted surface over the existing grid (option A), not cubes, not blobs</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Glowcap, moss canopy, fern coil, sprout coil in the library</t>
+          <t>One-block cells; detail is visual only</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>Outline 3</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -1193,37 +1209,37 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>W013</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Blocks &amp; art</t>
+          <t>World</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Parked decorative set: stained glass, porcelain floral, rune shrine</t>
+          <t>Smaller ground triangles near the player without hurting performance</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Dev pile; not this horizon</t>
+          <t>Subdivide only where it shows; set from preview-tool counts</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Foundations 4.1</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1235,7 +1251,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>W014</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1245,12 +1261,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>World / biome generation using the library blocks and props</t>
+          <t>Walk around: walk, sprint, crouch, jump, slide on facets</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1260,12 +1276,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>'Coming in the pipeline'; not started</t>
+          <t>Checklist T6</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Part II</t>
+          <t>Outline 5</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1277,17 +1293,17 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>W015</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Rendering</t>
+          <t>World</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Lighting, shadows, atmosphere, clouds, bloom, see-through blocks, glow light</t>
+          <t>Place and remove ground, one cell at a time, where the crosshair points</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1297,13 +1313,17 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Checklist T8</t>
+        </is>
+      </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>4.8-4.12</t>
+          <t>Outline 5</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1315,59 +1335,59 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>S016</t>
+          <t>W016</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Rendering</t>
+          <t>World</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Soft filtering / colour bleed / large-scale variation comparison</t>
+          <t>Seeded test landscape: meadow, dirt, stone, sand regions</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Owner picked D; colour bleed dropped after the playtest (halo). Variation + distance filtering kept (4.16)</t>
+          <t>Replaces the flat plain; versioned generator</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Outline 3</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>S017</t>
+          <t>W017</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Gameplay</t>
+          <t>Looks</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Movement: sprint, crouch, power slide</t>
+          <t>Textures and lighting carried over (sun, shadows, sky, fog, AO, bloom, glow)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1377,13 +1397,17 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Checklist T4</t>
+        </is>
+      </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>Outline D4</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1395,17 +1419,17 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>S018</t>
+          <t>W018</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Gameplay</t>
+          <t>Looks</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Block library + 10-slot hotbar</t>
+          <t>Smooth-filtered textures</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1415,13 +1439,13 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>Outline D8</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -1433,17 +1457,17 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>S019</t>
+          <t>W019</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Gameplay</t>
+          <t>Looks</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Debug time control (F8, [ ])</t>
+          <t>Natural blending between materials (height-based)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1453,13 +1477,17 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Checklist T3</t>
+        </is>
+      </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Part XV</t>
+          <t>Outline 4</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1471,64 +1499,64 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>S020</t>
+          <t>W020</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Looks</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Item logistics: pulse through pipes</t>
+          <t>Sky light: pits, overhangs and hollows go dark</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Built: harvester at a constant rate (faster under The Line); plain/clockwise/anticlockwise pipes give pulse spin; networks share out to stores (unlimited) and the machine; open ends fire straight, facing mouths catch; store view with bead heaps. Open: what harvesters draw from, what pulse becomes.</t>
+          <t>Checklist T5</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Part VI</t>
+          <t>Outline D4</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>S021</t>
+          <t>W021</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>First working machine (the placeholder becomes real)</t>
+          <t>Day-cycle music as in Voxistics</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -1538,54 +1566,54 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Core of the factory game. Logistics decided (pulse); waits on what pulse becomes / how it is burned</t>
+          <t>Checklist T10</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Part VI</t>
+          <t>Outline D2</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>S022</t>
+          <t>W022</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Byproducts and land health (industry safe when well run)</t>
+          <t>Footsteps on the beat, by gait and ground material</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Dev pile; core direction but not this horizon</t>
+          <t>Checklist T7</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Outline 5</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -1597,22 +1625,22 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>S023</t>
+          <t>W023</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Essence as a transmutation economy</t>
+          <t>Reactive sound effects that don't interfere with the music</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1622,96 +1650,92 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Candidate direction only</t>
+          <t>Checklist T9</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Part XIX</t>
+          <t>Outline D3</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>S024</t>
+          <t>W024</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Threat</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Ooze rifts born of neglect</t>
+          <t>Effects on their own thread, with a voice cap</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Dev pile</t>
+          <t>So busy moments never click or cut out</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Outline D3</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>S025</t>
+          <t>W025</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Fluids</t>
+          <t>First person only</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Dev pile; heavy</t>
-        </is>
-      </c>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n"/>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Outline D9</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -1723,327 +1747,327 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>S026</t>
+          <t>W026</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Vapours and gases</t>
+          <t>Raw mouse input</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Dev pile; heavy</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Engine review 2.7</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>S027</t>
+          <t>W027</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Plants drop when their support is removed</t>
+          <t>Hotbar and material library carried over</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Dev pile</t>
-        </is>
-      </c>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Part XX</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>S028</t>
+          <t>W028</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Menus</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Day-cycle music (one clock)</t>
+          <t>Title, slots, pause, options (look, graphics, display, audio, keys, accessibility), saves</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr"/>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Carried over; checklist T11</t>
+        </is>
+      </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Part XIV</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>S029</t>
+          <t>W029</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Debug &amp; checks</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>World sound palette + three soundscape axes</t>
+          <t>Screenshot key</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Owner finds it plain; develop later</t>
+          <t>M0; for comparing builds</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Foundations 7</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>S030</t>
+          <t>W030</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Debug &amp; checks</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Develop the palette's character further</t>
+          <t>MinGW cross-compile and shader check set up here</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>When the game's direction is clearer</t>
+          <t>Tools being installed</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Foundations 7</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>S031</t>
+          <t>W031</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Debug &amp; checks</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Machine sounds react to the placeholder machine</t>
+          <t>CPU still-image preview of faceted ground (with triangle counts)</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>Online on placing; hum and rhythm near machines</t>
+          <t>M1's first deliverable</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Foundations 4.1</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>S032</t>
+          <t>W032</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Debug &amp; checks</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Positional (stereo) sound</t>
+          <t>Release performance check on the owner's PC (Ctrl+F3 report)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Owner: go ahead. Placed sounds pan, ping-pong echo, Mono audio toggle</t>
+          <t>Awaits the owner at each milestone</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>Foundations 7</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>S033</t>
+          <t>W033</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Sounds waiting on systems: mending, rift closed, rift omens</t>
+          <t>New CLAUDE.md, DESIGN.md and DECISIONS.md; Voxistics docs archived</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Won't</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Built and tested; nothing triggers them yet</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Foundations 6</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -2055,159 +2079,159 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>S034</t>
+          <t>W034</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>The Line</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>The Line prototype: travelling pivot, clockwise spin, time expression</t>
+          <t>Split game.cpp into input, menus, hud</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Should</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Playtest fixes: pivot now lands on the spot you actually spend time in x and z (16-block cells remembering where their time was spent; 30-min half-life). Expression (owner's pick): the visible sky races ahead near the line and runs slow after you leave; sun and light keep the real clock; wobble kept faint.</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Part XVIII</t>
+          <t>Engine review 2.7</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>S035</t>
+          <t>W035</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>The Line</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Hide the debug marker once the sky effect is signed off</t>
+          <t>Third person and an animated player model</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr"/>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>If wanted</t>
+        </is>
+      </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Part XVIII</t>
+          <t>Outline D9</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>S036</t>
+          <t>W036</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>The Line</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Player structures as extra pivot sources</t>
+          <t>Death metal music</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Parked</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Owner expected the essence attractor to do this; today it doesn't (it only draws from convergence zones). Owner to decide whether attractors should pull The Line's pivot.</t>
+          <t>Real instruments are hard to emulate</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Part XVIII</t>
+          <t>Outline D2</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>S038</t>
+          <t>W037</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Standing rules</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Nothing anyone owns: no brands, currencies, crypto, borrowed art or names</t>
+          <t>Action systems: enemies, projectiles, particles, with budgets</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>Standing rule</t>
-        </is>
-      </c>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n"/>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Part VIII</t>
+          <t>Outline 2</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -2219,37 +2243,33 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>S039</t>
+          <t>W038</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Standing rules</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Photosensitivity: nothing flashes more than 3 times a second</t>
+          <t>Real terrain generator with caves</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>Standing rule</t>
-        </is>
-      </c>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n"/>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Part XI</t>
+          <t>Outline 2</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -2261,37 +2281,37 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>S040</t>
+          <t>W039</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Vocal ad-libs and footfalls</t>
+          <t>Unsupported ground falls (Voxistics gravity)</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Parked</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Owner: keep</t>
+          <t>Revisit after the first test</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
@@ -2303,17 +2323,17 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>S041</t>
+          <t>W040</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>'Unveil' cue on first placement of a block type</t>
+          <t>Covered grass dies back to dirt</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2328,12 +2348,12 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Owner: nixed; the recipe stays unused</t>
+          <t>Revisit after the first test</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
@@ -2345,37 +2365,37 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>S042</t>
+          <t>W041</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Footsteps on the beat, by gait and ground hardness</t>
+          <t>Plants that turn to face you</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Parked</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Crouch/walk/sprint; soft scuffs, hard knocks in key</t>
+          <t>Revisit after the first test</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
@@ -2387,964 +2407,320 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>S043</t>
+          <t>W042</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>World</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Default plain as a fractal patchwork of three ground materials</t>
+          <t>See-through materials (glass, ice, water)</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>Grass / sand / pebbles by feel underfoot; flat v2; materials swappable</t>
-        </is>
-      </c>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n"/>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Part II</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>S044</t>
+          <t>W043</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Buttons that look and feel pressable (mechanical press cue)</t>
+          <t>Colour-vision modes; first-steps tutorial</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Parked</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Keys act on release; sliders are beads on a string</t>
+          <t>Served Voxistics features</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Part XII</t>
+          <t>Outline 7</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>S045</t>
+          <t>W044</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Standing rules</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Privacy: no telemetry, crash reporting or hardware reading; target a modest old Windows PC</t>
+          <t>Gamepad support</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Must</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Standing rule</t>
-        </is>
-      </c>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n"/>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Engine review 2.7</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude (proposed)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>S046</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>Crafting</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="inlineStr">
-        <is>
-          <t>Crafting system brainstorm: gathering, representation, uses, advancement from the natural surroundings</t>
-        </is>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>After the playtest. Seed: microbes/germs gathered as essence, coloured/'flavoured' by the source's biological makeup. Owner to confirm priority.</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>Part XX</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>S047</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>Playtest fixes</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>Footsteps louder; fog haze + distance filtering; midday hitch (music slices, sliced shadow redraw)</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>From the first playtest on the owner's rig</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>4.8, 4.16, 14.7</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A47" s="6" t="n"/>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>S048</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>Forgiving power-slide timing; faster sprint (7.5)</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>Crouch/sprint in either order within 0.3-0.4 s</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>4.7</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A48" s="6" t="n"/>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>S049</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Rendering</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>Frame rate limit 30-200 (default 60) and vsync toggle</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>Graphics settings</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>12.y</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A49" s="6" t="n"/>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>S050</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Breaking blocks: how it is done, and with what tools (if any)</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Could</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>Parked</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>Owner: comes later, once we decide what tools there are. Today a click breaks a block instantly. Priority is the owner's to set.</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>Part XX</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>Claude (proposed)</t>
-        </is>
-      </c>
+      <c r="A50" s="6" t="n"/>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="6" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>S051</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Rendering</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>Pre-generated fracture: a broken block splits into pieces that tumble and settle</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>Could</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>Parked</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>Owner's idea, for with S050. Cheap by design: fracture patterns baked once per shape (a handful of variants), a few short-lived pieces per break, no per-block data. Nothing flashes.</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>Part XX</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>Claude (proposed)</t>
-        </is>
-      </c>
+      <c r="A51" s="6" t="n"/>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="6" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>S052</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>Translation / language packs</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Won't</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>Owner: not a priority; English only, kept minimal so non-native speakers pick it up through play. Estimate if ever wanted: Latin scripts a few days (string table, accented glyphs); CJK needs a glyph cache.</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A52" s="6" t="n"/>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>S053</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Art</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>A big new batch of library blocks to sort through</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>36 trial materials in the library (batch_sept.vtex), four families; waiting on the owner's sort</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>4.13, 4.15</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A53" s="6" t="n"/>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>S054</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Reviews: music fit; optimisation and architecture; texture library direction</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>docs/REVIEW_2026-09.md; perf fixes merged, proposals await the owner</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A54" s="6" t="n"/>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="6" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>S055</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>Pulse spin: three pipe kinds, spin carried and counted</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>Owner's idea; seen as corkscrew comets in the air and heaps by colour in stores</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A55" s="6" t="n"/>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>S056</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>Fliers: two-winged day-lived creatures that fly low; the line ages them</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>Owner's idea. Die after one game day or sooner under The Line; death makes grass glow vividly for a while, or grows mold on dirt/wood</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>Part XXI</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A56" s="6" t="n"/>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>S057</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>Mold that sprouts a mushroom after a game day or after rain</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Could</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>Owner's idea; rain needs a weather system (to discuss)</t>
-        </is>
-      </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr">
-        <is>
-          <t>Claude (proposed)</t>
-        </is>
-      </c>
+      <c r="A57" s="6" t="n"/>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
+      <c r="F57" s="6" t="n"/>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="6" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>S058</t>
-        </is>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>Covered grass turns to dirt (not overnight)</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>Deprived of sky, not of daylight</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>Part V</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A58" s="6" t="n"/>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="6" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>S059</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>Weather (rain first)</t>
-        </is>
-      </c>
-      <c r="D59" s="6" t="inlineStr">
-        <is>
-          <t>Could</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>Owner: yet to discuss</t>
-        </is>
-      </c>
-      <c r="G59" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="6" t="inlineStr">
-        <is>
-          <t>Claude (proposed)</t>
-        </is>
-      </c>
+      <c r="A59" s="6" t="n"/>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="6" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="6" t="n"/>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="6" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>S060</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>The Line</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>The Line grows to a plane with the player's power and influence</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Won't</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>Owner: low priority, discuss later</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Part XVIII</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A60" s="6" t="n"/>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="6" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="6" t="n"/>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="6" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>S061</t>
-        </is>
-      </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="C61" s="6" t="inlineStr">
-        <is>
-          <t>Diffuser: spends pulse widening The Line's band (the first loop)</t>
-        </is>
-      </c>
-      <c r="D61" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="inlineStr">
-        <is>
-          <t>Owner's design: feed per second keeps the band wide; harvesters above/below need it</t>
-        </is>
-      </c>
-      <c r="G61" s="6" t="inlineStr">
-        <is>
-          <t>6.0, XVIII</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A61" s="6" t="n"/>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="6" t="n"/>
+      <c r="F61" s="6" t="n"/>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="6" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>S062</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>First-steps tutorial on a new world, skippable</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>One line at a time, moves on as done; Enter skips</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A62" s="6" t="n"/>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="6" t="n"/>
+      <c r="G62" s="6" t="n"/>
+      <c r="H62" s="6" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>S063</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>New world starts with harvester, pipe, chest, diffuser on the hotbar</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr"/>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A63" s="6" t="n"/>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="6" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="6" t="n"/>
+      <c r="F63" s="6" t="n"/>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="6" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>S064</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>Colour-vision modes, one per kind of colour blindness</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>Accessibility &gt; Colour vision: 5 modes for the pulse colours; tested with dichromat simulations (the big win: no-colour, where blue and red merged)</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>11.x</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A64" s="6" t="n"/>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="6" t="n"/>
+      <c r="H64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>S065</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>Machines sped up or slowed by time flux</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Could</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>Owner: pipes and pulse in the air stay unaffected; harvesters are the first</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+      <c r="A65" s="6" t="n"/>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n"/>

</xml_diff>

<commit_message>
Record D16 (draw only what's seen, load ahead) and start M0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -809,7 +809,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -2523,14 +2523,46 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
-      <c r="D46" s="6" t="n"/>
-      <c r="E46" s="6" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
-      <c r="H46" s="6" t="n"/>
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>W045</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Render only what can be seen; preload what may be seen soon</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>Frustum culling exists; hidden-chunk skipping and heading-aware loading in M1</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Foundations 4.3</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>

</xml_diff>

<commit_message>
M0.3: walkgrid DESIGN.md, Voxistics docs archived, CLAUDE.md draft
DESIGN.md keeps the engine parts with their Voxistics section numbers,
so code references still resolve; Voxistics-only parts are archived in
docs/voxistics/DESIGN.md. Part I is rewritten so the seed-file rule
can't be read as a rule against carrying the engine. The new CLAUDE.md
is in docs/CLAUDE_DRAFT.md for the owner's review; it replaces
CLAUDE.md only once approved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -977,12 +977,12 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Approved with the foundations</t>
+          <t>tools/check_layers.py reports 16 violations, removed by M0 steps</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -1889,12 +1889,12 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>M0; for comparing builds</t>
+          <t>F2; built, awaiting the owner's check on Windows</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Tools being installed</t>
+          <t>tools/check_mingw.sh; shader check runs clean</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2057,12 +2057,12 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>DESIGN.md carried over; CLAUDE.md drafted, awaiting the owner</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
M0.3: approved CLAUDE.md replaces the Voxistics one
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2057,12 +2057,12 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>DESIGN.md carried over; CLAUDE.md drafted, awaiting the owner</t>
+          <t>CLAUDE.md and DESIGN.md done; DECISIONS.md done</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Log decisions D20-D27 and update the rules
D20 graphics minimum to FL 11.0 / SM 5.0 (M0 step 0.16). D21 harmless
reads of OS limits only, never kept or shown. D22 no finer sculpting for
now. D23 no online play. D24 flash limit and accessibility no longer
standing rules. D25 synthesized sound only (hard rule). D26 text must be
translatable (M1 step 0). D27 SOP approved and binding with two tiers;
engine-to-game hooks capped and listed (FOUNDATIONS.md 2.1).

CLAUDE.md, SOP, FOUNDATIONS, DESIGN, GOALS, ROADMAP, M0 plan, forecasts
(new F16) and the scope sheet updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2470,7 +2470,7 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Served Voxistics features</t>
+          <t>Served Voxistics features; accessibility no longer a standing rule (D24)</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2565,64 +2565,256 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
-      <c r="H47" s="6" t="n"/>
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>W046</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Graphics minimum: Direct3D feature level 11.0, shader model 5.0</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>M0.16 (D20)</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D20</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>W047</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Harmless reads of OS limits only (thread count, video-memory budget); never kept or shown</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Standing rule (D21)</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D21</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="6" t="n"/>
-      <c r="D49" s="6" t="n"/>
-      <c r="E49" s="6" t="n"/>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="6" t="n"/>
-      <c r="H49" s="6" t="n"/>
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>W048</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>No online play, no network code</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Standing rule, never 'done' (D23)</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D23</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="6" t="n"/>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>W049</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Sound</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Synthesized sound only: no recorded or sampled audio</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Standing rule, never 'done' (D25)</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D25</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="6" t="n"/>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="6" t="n"/>
-      <c r="H51" s="6" t="n"/>
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>W050</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Menus</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Text ready for any language: string table, wider font atlas</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>M1 step 0 (D26)</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D26</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="6" t="n"/>
-      <c r="D52" s="6" t="n"/>
-      <c r="E52" s="6" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
-      <c r="H52" s="6" t="n"/>
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>W051</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>SOP binding, two tiers; hooks capped and listed</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>docs/SOP.md; FOUNDATIONS.md 2.1 (D27)</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D27</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>

</xml_diff>

<commit_message>
M0.16: graphics minimum raised to feature level 11.0, shader model 5.0
Feature card (SOP): opens tessellation and compute shaders for M1 and
later (D20); no visual change. Files: render.cpp (device asks for 11.0
only; all 13 shaders compile as vs_5_0/ps_5_0), main.cpp (a message box
instead of a silent exit when the device can't be made). Cost: none;
the shader cache recompiles once, since the profile is part of each
shader's key. The message box text is a literal until M1's string table
(D26).

Checked here: native tests, shaders (glslang), MSVC check, MinGW build,
layers. Not checked: that D3DCompile accepts every shader at 5_0 (it
only runs on Windows; SM5 is a superset of SM4, so expected).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Frames before and after must match, minus removed features</t>
+          <t>M0 steps done; awaiting the owner's Windows build and checklist</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Checklist T12, T13</t>
+          <t>Interpolated rendering in M0.12; frame cap only with vsync off</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M0.10</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -1103,12 +1103,12 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Approved with the foundations</t>
+          <t>M0.13, with a native test</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1767,12 +1767,12 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M0.14; awaiting the feel check (C5)</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2099,12 +2099,12 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M0.11</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2587,12 +2587,12 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>M0.16 (D20)</t>
+          <t>M0.16; awaiting the Windows build to confirm D3DCompile accepts SM5</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Footsteps louder and brighter (D29); materials from the library (D30)
Footfall base level -29 to -13 and the soft-ground low-pass floor
700 to 1100 Hz: the owner's pick of three mixed clips. The palette's
-21 dB ceiling clamps most of the raise (about +5 dB peak), which is
why every clip sounded subtle; lifting it for footsteps is put to the
owner in M1 step 1.1. The existing "works" BRIGHT flag in the sound
analysis was there before this change.

Materials are chosen from the library menu; the hotbar stays as a
placeholder. M1 plan, decisions and scope rows W003, W022, W027 updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>M0 steps done; awaiting the owner's Windows build and checklist</t>
+          <t>M0 done, run on the owner's machine 2026-09-25</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Checklist T7</t>
+          <t>Checklist T7. Louder and brighter (D29); still subtle, owner decides the ceiling in M1 step 1.1</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Hotbar and material library carried over</t>
+          <t>Choose materials from the library menu; hotbar kept for now</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1812,15 +1812,19 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="F28" s="6" t="n"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Owner (D30): materials are chosen in the library. The hotbar stays as a placeholder, possibly for other GUI later</t>
+        </is>
+      </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Outline 7</t>
+          <t>Decisions D30</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M1.1: sound effects render on their own thread
The world sound palette rendered on the main thread and spiked to
14.9 ms in the M0 baseline (forecast F11). It now renders on a worker,
like the music: the main thread posts cues, releases and fades to a
fixed 64-entry mailbox and the latest state (axes, scene, listener,
gait) under a brief lock. XAudio2's buffer-end callback wakes the
worker; it sleeps when silent. Three buffers (~35 ms) stay queued, one
more after any underrun, up to 8. Same calls in audio.h.

The 48-voice cap with priority tiers already existed; a new test floods
the palette and checks it holds and that an interaction still sounds.
Stress render: 0.6 ms median, 1.1 ms p95 per 11.6 ms buffer at the cap.

Plan approved (D32). Feature card in M1_PLAN; DESIGN 10.1/10.4, cost
ledger, F11 and scope W024 updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -1687,12 +1687,12 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>So busy moments never click or cut out</t>
+          <t>Built in M1.1 (own thread, mailbox, 48-voice cap tested); awaiting the owner's Ctrl+F3 report</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">

</xml_diff>

<commit_message>
M1.3: twelve starting materials, chosen on contact sheets
The preview tool gains a contact-sheet mode (facet_preview.sh OUTDIR
sheets): every natural candidate on a faceted mound with a cliff under
a low sun, then each pair of the picks meeting. Picks (D36, provisional
while the owner is away, D33): meadow grass, dry turf, moss, dirt,
loam, clay, sand, gravel, stone, slate, sandstone, snow. Sheets in
docs/pictures/m1_3. TEXTURE_BRIEF.md rewritten for faceted, smoothly
filtered, world-projected ground (tops and sides, height maps drive
borders). Parking the unpicked textures moves to 1.9, when the old
roster that still uses them goes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2821,14 +2821,46 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="6" t="n"/>
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>W052</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Twelve starting materials, chosen on contact sheets</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>D36, provisional until the owner confirms; docs/pictures/m1_3</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Decisions D36</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>

</xml_diff>

<commit_message>
M1.10: text for any language (string table)
Every player-facing word moves to assets/text/en.txt (D26, D42): a
key = text table in UTF-8, English under the chosen language
(language= in settings.cfg), {n} slots, "[key]" for a missing one.
strtable.cpp/.h (layer 2) loads it; menus, HUD, toasts, key names and
the start-up message read it. The UI atlas bakes ASCII, Latin-1 and the
table's other letters in the table's named font; row labels and titles
shrink to fit. tools/check_strings.py (run by tests/run.sh) fails on
words left in game code, undefined or unused keys, and mismatched
slots; --pseudo writes the test language (assets/text/test.txt). Debug
aids stay English, marked. FindAssetDirectory is shared by textures and
text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2763,12 +2763,12 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>M1 step 0 (D26)</t>
+          <t>M1 step 1.10 (D26, D42): assets/text, strtable.*, atlas from the table, check_strings.py. Awaiting the owner's check (test language)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">

</xml_diff>

<commit_message>
M1.11: draw only what's seen; load ahead
Each chunk's mesh job records which of its sides see each other through
open cells (FacetOpenings). Each frame a walk outward from the camera's
chunk, through those openings and the frustum, never back toward the
camera, marks what could be seen; chunks in view it never reaches are
sealed off by ground and aren't drawn (F3: CHUNKS HIDDEN). The shadow
pass is unchanged. Columns and meshes queue by distance weighted by the
heading (look pulled toward movement), nearest nine columns first; a
turn past 45 degrees re-orders the queue. Tested: no eye ray meets
ground in a skipped chunk, from the surface or a sealed tunnel (D43).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2553,12 +2553,12 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>Frustum culling exists; hidden-chunk skipping and heading-aware loading in M1</t>
+          <t>Frustum culling; hidden-chunk skipping and heading-aware loading built in M1 step 1.11 (D43). Awaiting a Ctrl+F3 report (CHUNKS HIDDEN)</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">

</xml_diff>

<commit_message>
M1.12: footstep clips past the ceiling; sand's step; M1 review docs
The synth can hold footsteps to their own ceiling (SetFootstepCeiling);
the game keeps -21 dB until the owner picks from clips made by the new
`tools/sound_demo.sh steps OUTDIR` (grass, stone and sand over the
midday music at -21, -16 and -11 dB). Sand gets its own sound material,
a soft bright hiss where soils crunch (provisional, D44).

Docs: the T1-T13 checklist with what was checked here and what waits
for the owner (M1_PLAN 1.12), the M1 reflection, the forecast review
(and F20), scope rows, SOUND_PALETTE R1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -1397,12 +1397,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Checklist T4</t>
+          <t>Carried over and building; awaiting the owner's checklist T4 (M1.12)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Checklist T10</t>
+          <t>Carried over and building; awaiting the owner's checklist T10 (M1.12)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Checklist T7. Louder and brighter (D29); still subtle, owner decides the ceiling in M1 step 1.12 (D31)</t>
+          <t>Checklist T7. Louder and brighter (D29). Clips at three footstep ceilings made in M1.12 (D44); the game stays at -21 dB until the owner picks</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Checklist T9</t>
+          <t>Carried over and building; awaiting the owner's checklist T9 (M1.12)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Carried over; checklist T11</t>
+          <t>Carried over and building; awaiting the owner's checklist T11 (M1.12)</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2867,14 +2867,46 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="6" t="n"/>
-      <c r="D54" s="6" t="n"/>
-      <c r="E54" s="6" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
-      <c r="H54" s="6" t="n"/>
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>W053</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Sound</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Sand sounds like sand underfoot (its own soft hiss)</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>Added in M1.12 so T7's four grounds differ (D44); owner to keep or drop</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Sound palette R1</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>

</xml_diff>

<commit_message>
Project notes: a full write-up for the owner and any agent
docs/PROJECT_NOTES.md: what walkgrid is and what makes it its own
(D60), the working rules in short, where everything lives, what's built
through D60 and what hasn't been seen running, the code by layer and
the life of a frame and a chunk, how to build and check, the plug-in
points for adding content without engine changes, the pitfalls that
have bitten us, and what's next -- including small tasks a helper agent
could take on. Listed in docs/README.md. Scope: weather (Could, later).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2894,7 +2894,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Added in M1.12 so T7's four grounds differ (D44); owner to keep or drop</t>
+          <t>Added in M1.12 so T7's four grounds differ (D44); waits until the owner can hear footsteps (D48)</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -2909,14 +2909,46 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="6" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>W054</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Weather: kinds of weather orchestrated by a weather state that sets the sky, cloud, fog, light and sound knobs; cheap tricks only, nothing volumetric</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>Later (owner, D58/D59). The cloud layers and jet stream are its first knobs. Design notes are a helper-agent task (PROJECT_NOTES 9)</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN Part XIII</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>

</xml_diff>

<commit_message>
Park the terracing (D62): back burner until a nicer way
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2951,14 +2951,46 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n"/>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="6" t="n"/>
-      <c r="D56" s="6" t="n"/>
-      <c r="E56" s="6" t="n"/>
-      <c r="F56" s="6" t="n"/>
-      <c r="G56" s="6" t="n"/>
-      <c r="H56" s="6" t="n"/>
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>W055</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Gentle slopes roll instead of terracing, with player edits kept crisp</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Won't</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>D62: back burner until a nicer way. FacetShape::terrace is built but off (it softens one-cell edits)</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 23.1</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>

</xml_diff>

<commit_message>
docs/AGENT_TASKS.md: 30 tasks for a helper agent between sessions
For the days without Claude: how to work (a branch per task, the checks,
the report template), what's off limits (threads, the renderer's
structure, saves, terrain output, sound recipes, decisions, reference),
and 30 tasks in seven groups: checks and tidying, tests for pure code,
tools, content through the plug-in points, small features, research
notes for the next session (lighting, weather, terracing, our own look,
caves, M2), and review. Linked from PROJECT_NOTES and docs/README.
Scope: W032 done (the owner's two reports).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2023,12 +2023,12 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Awaits the owner at each milestone</t>
+          <t>Two Ctrl+F3 reports from the owner, 2026-09-26 (199 fps, no hitches): docs/COST_LEDGER.md</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fill light: shade keeps its shape (D63)
The world shader adds light the sun puts into the air and onto the ground
around: the sky brighter on the side toward the sun, and a warm bounce
from sunlit ground onto faces tilting sideways or down. Shade's sky light
is a quarter greyer. Scaled by the baked sky view and openness; two dot
products per pixel, no pass. The preview renderer mirrors it and gains
two low-sun views. Pictures in docs/pictures/fill_light (top before,
bottom after). DESIGN 4.9, D63, scope W056.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2993,14 +2993,46 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="6" t="n"/>
-      <c r="H57" s="6" t="n"/>
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>W056</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Shadowed ground keeps its shape: fill light (brighter sky toward the sun, warm bounce from sunlit ground), shadow less blue</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>D63; replaces what screen-space AO was faking, without the golf-ball dimples. Awaiting the owner's look in game</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.9</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n"/>

</xml_diff>

<commit_message>
F2 screenshots no longer stall the game
The owner's performance report showed 70-100 ms hitches with no system
named: the PNG encode ran on the frame F2 was pressed. It now runs on a
job thread (new channel JOB_FILES); the frame only reads the picture
back, and the toast follows once the file is on disk. Scope W057.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3035,14 +3035,46 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="n"/>
-      <c r="B58" s="6" t="n"/>
-      <c r="C58" s="6" t="n"/>
-      <c r="D58" s="6" t="n"/>
-      <c r="E58" s="6" t="n"/>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="6" t="n"/>
-      <c r="H58" s="6" t="n"/>
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>W057</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>F2 screenshots without a stall: the PNG is encoded on a job thread</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>The owner's report showed 70-100 ms hitches from F2; now only the read-back runs on the frame. Toast when on disk</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 7.2.1</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>

</xml_diff>

<commit_message>
Distant ground less white (D64)
The loaded world's edge fades over its last fifth (was 30%), and the
ground's fog takes only a quarter of the sky's glow around the sun, which
turned hills toward the sun white. Preview mirrors it; picture in
docs/pictures/fog (top before, bottom after). Scope W058.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3077,14 +3077,46 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="6" t="n"/>
-      <c r="D59" s="6" t="n"/>
-      <c r="E59" s="6" t="n"/>
-      <c r="F59" s="6" t="n"/>
-      <c r="G59" s="6" t="n"/>
-      <c r="H59" s="6" t="n"/>
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>W058</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Distant ground keeps its colour: narrower edge fade, no sun glow in the ground's fog</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>D64. The real fix for seeing far is cheap distant ground (a far, coarse ring): a future plan</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.9</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="n"/>

</xml_diff>

<commit_message>
Plan notes from the third play-test (docs/PLAN_LOOK.md)
Causes found in the code for what the owner saw (frozen clouds, ray-like
streaks, the orange lines being the material blend, per-block texture
repetition), the look and sky plan A-H, open questions, and the parked
building layer (owner's idea). Scope rows W059-W067. Planning only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3119,94 +3119,382 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="6" t="n"/>
-      <c r="D60" s="6" t="n"/>
-      <c r="E60" s="6" t="n"/>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="6" t="n"/>
-      <c r="H60" s="6" t="n"/>
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>W059</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Sky</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Clouds that live: faster drift, shapes that form, stretch and break up downwind</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK A; waits for the owner's go</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.9</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="6" t="n"/>
-      <c r="D61" s="6" t="n"/>
-      <c r="E61" s="6" t="n"/>
-      <c r="F61" s="6" t="n"/>
-      <c r="G61" s="6" t="n"/>
-      <c r="H61" s="6" t="n"/>
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>W060</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Sky</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>High streaks shorter and patchy, no ray-like convergence toward the sun</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK B</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.9</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n"/>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
-      <c r="E62" s="6" t="n"/>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="n"/>
-      <c r="H62" s="6" t="n"/>
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>W061</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Sky</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Low clouds soft-edged and rim-lit, never flat puddles</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK C</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.9</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n"/>
-      <c r="B63" s="6" t="n"/>
-      <c r="C63" s="6" t="n"/>
-      <c r="D63" s="6" t="n"/>
-      <c r="E63" s="6" t="n"/>
-      <c r="F63" s="6" t="n"/>
-      <c r="G63" s="6" t="n"/>
-      <c r="H63" s="6" t="n"/>
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>W062</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Clean material edges: a smooth noise-driven blend band, no thin streaks of one material in another</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK D; the orange lines at the slate ridge</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 23.4</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n"/>
-      <c r="B64" s="6" t="n"/>
-      <c r="C64" s="6" t="n"/>
-      <c r="D64" s="6" t="n"/>
-      <c r="E64" s="6" t="n"/>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="6" t="n"/>
-      <c r="H64" s="6" t="n"/>
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>W063</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Textures without visible repetition: per-cell random shift and turn, and large-scale patches per material</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK E</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.16</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="6" t="n"/>
-      <c r="H65" s="6" t="n"/>
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>W064</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>64-pixel material textures</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK F; density to be decided by the owner</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>TEXTURE_BRIEF</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n"/>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="6" t="n"/>
-      <c r="D66" s="6" t="n"/>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
-      <c r="H66" s="6" t="n"/>
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>W065</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Debug views: baked darkening only, shadows only, materials only</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK G; to find the patches seen at noon</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN Part XVI</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n"/>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="6" t="n"/>
-      <c r="D67" s="6" t="n"/>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="6" t="n"/>
-      <c r="H67" s="6" t="n"/>
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>W066</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>Looks</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Slate lighter and less saturated</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>PLAN_LOOK H</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>TEXTURE_BRIEF</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="n"/>
-      <c r="B68" s="6" t="n"/>
-      <c r="C68" s="6" t="n"/>
-      <c r="D68" s="6" t="n"/>
-      <c r="E68" s="6" t="n"/>
-      <c r="F68" s="6" t="n"/>
-      <c r="G68" s="6" t="n"/>
-      <c r="H68" s="6" t="n"/>
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>W067</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>A building layer: crisp placed blocks that sit on the faceted ground in a satisfying way</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Won't</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>Owner's idea, 2026-09-26; questions in PLAN_LOOK. The Voxistics cube mesher and pieces were removed in M1.9 (D41)</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.15</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n"/>

</xml_diff>

<commit_message>
Cloud research; 64-pixel textures (D65); research standard (D66)
docs/research/CLOUDS.md: how real cumulus and cirrus move and change,
from agency and peer-reviewed sources (read via search summaries; to be
checked at the source), what that means as angular speed on screen, why
ours look frozen, and proposed targets. D65: textures 64 px per block.
D66: reliable sources only, in CLAUDE.md and the helper Brief.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3146,7 +3146,7 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>PLAN_LOOK A; waits for the owner's go</t>
+          <t>PLAN_LOOK A; researched in docs/research/CLOUDS.md; real or compressed time is the owner's call</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>PLAN_LOOK F; density to be decided by the owner</t>
+          <t>PLAN_LOOK F; 64 pixels per block (D65)</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grok translations: East Asian and African languages (T18-T33)
Japanese, Simplified and Traditional Chinese, Korean, Vietnamese,
Indonesian, Filipino, Malay, Swahili, Hausa, Yoruba, Zulu, Xhosa,
Afrikaans, Somali, Amharic. Each pack says what the text system can
draw today: any code point the font has, one cell wide, no stacked
marks. Scope W068 (wide characters, planned) and W069 (shaping and
stacked marks, parked); noted in PLAN_TUESDAY.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3497,24 +3497,88 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="n"/>
-      <c r="B69" s="6" t="n"/>
-      <c r="C69" s="6" t="n"/>
-      <c r="D69" s="6" t="n"/>
-      <c r="E69" s="6" t="n"/>
-      <c r="F69" s="6" t="n"/>
-      <c r="G69" s="6" t="n"/>
-      <c r="H69" s="6" t="n"/>
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>W068</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>East Asian text: double-width glyph cells in the UI atlas and layout, for Chinese, Japanese and Korean</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>Owner: be inclusive of Asian and African languages. Translations T18-T21 (and Amharic, T33, if its script is wide) wait on it. Fonts per language via the font line</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.6.2</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n"/>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="6" t="n"/>
-      <c r="D70" s="6" t="n"/>
-      <c r="E70" s="6" t="n"/>
-      <c r="F70" s="6" t="n"/>
-      <c r="G70" s="6" t="n"/>
-      <c r="H70" s="6" t="n"/>
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>W069</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Scripts that need shaping or stacked marks (Devanagari, Thai, Arabic right-to-left, combining tone marks as in some Yoruba)</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>Won't</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>A per-glyph atlas can't join or reorder letters; needs a shaping step. Kept so it isn't forgotten</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 4.6.2</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n"/>

</xml_diff>

<commit_message>
Appraise E14-E16 (ChatGPT): durable saves gap found; footstep timing question
E15 surfaced that saves aren't flushed to disk before the swap and that
loading never falls back to the .bak: scope W070, added to Tuesday's
batch 1. E14 raised stride- vs beat-timed footsteps (owner's call) and
modal dig/place sounds. E16 confirmed our loop's overload policy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CTkmAJqE7SezZyw5ooiXgA
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3581,14 +3581,46 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="n"/>
-      <c r="B71" s="6" t="n"/>
-      <c r="C71" s="6" t="n"/>
-      <c r="D71" s="6" t="n"/>
-      <c r="E71" s="6" t="n"/>
-      <c r="F71" s="6" t="n"/>
-      <c r="G71" s="6" t="n"/>
-      <c r="H71" s="6" t="n"/>
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>W070</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Durable saves: flush the new file to disk before swapping it in, load the .bak when the main save is missing or damaged, and test every interruption point</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>From Grok/ChatGPT E15 (docs/grok_reviews/round2_E_part2.md): today safe against a game crash, not a power cut, and LoadGame never tries the .bak</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>DESIGN 7.3</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n"/>

</xml_diff>